<commit_message>
로봇 자동 갱신: 2026-05-23
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8017" uniqueCount="3985">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8021" uniqueCount="3987">
   <si>
     <t>연번</t>
   </si>
@@ -3662,12 +3662,12 @@
     <t>조선백호</t>
   </si>
   <si>
+    <t>인천광역시 중구 개항로96번길 11(1,2층 경동)</t>
+  </si>
+  <si>
     <t>인천광역시 중구 개항로96번길 11(1층 경동)</t>
   </si>
   <si>
-    <t>인천광역시 중구 개항로96번길 11(1,2층 경동)</t>
-  </si>
-  <si>
     <t>주윤 상차림</t>
   </si>
   <si>
@@ -3809,12 +3809,12 @@
     <t>그리너리 바스켓</t>
   </si>
   <si>
+    <t>인천광역시 중구 백운로 510(1동 지1층 운북동)</t>
+  </si>
+  <si>
     <t>인천광역시 중구 백운로 510(2동 1,2층 운북동)</t>
   </si>
   <si>
-    <t>인천광역시 중구 백운로 510(1동 지1층 운북동)</t>
-  </si>
-  <si>
     <t>꿈꾸는카페-혜윰도그파크점</t>
   </si>
   <si>
@@ -4007,12 +4007,12 @@
     <t>송경솥밥</t>
   </si>
   <si>
+    <t>광주광역시 동구 동명로14번길 19-8(2층 동명동)</t>
+  </si>
+  <si>
     <t>광주광역시 서구 상무시민로 136(수성빌딩 1층 치평동)</t>
   </si>
   <si>
-    <t>광주광역시 동구 동명로14번길 19-8(2층 동명동)</t>
-  </si>
-  <si>
     <t>쉘터커피로스터스</t>
   </si>
   <si>
@@ -9600,6 +9600,12 @@
   </si>
   <si>
     <t>경상남도 거제시 장목면 거제북로 1073(1층)</t>
+  </si>
+  <si>
+    <t>워크오프(work off)</t>
+  </si>
+  <si>
+    <t>경상남도 양산시 물금읍 화합3길 16(101호)</t>
   </si>
   <si>
     <t>이시마표고버섯식당농원</t>
@@ -39544,7 +39550,7 @@
         <v>1616.0</v>
       </c>
       <c r="B1617" t="s" s="3">
-        <v>892</v>
+        <v>3212</v>
       </c>
       <c r="C1617" t="s" s="2">
         <v>6</v>
@@ -39553,7 +39559,7 @@
         <v>3044</v>
       </c>
       <c r="E1617" t="s" s="3">
-        <v>3212</v>
+        <v>3213</v>
       </c>
     </row>
     <row r="1618" ht="36.0" customHeight="true">
@@ -39561,7 +39567,7 @@
         <v>1617.0</v>
       </c>
       <c r="B1618" t="s" s="3">
-        <v>3213</v>
+        <v>892</v>
       </c>
       <c r="C1618" t="s" s="2">
         <v>6</v>
@@ -40193,7 +40199,7 @@
         <v>3287</v>
       </c>
       <c r="C1655" t="s" s="2">
-        <v>580</v>
+        <v>6</v>
       </c>
       <c r="D1655" t="s" s="2">
         <v>3044</v>
@@ -40675,7 +40681,7 @@
         <v>3044</v>
       </c>
       <c r="E1683" t="s" s="3">
-        <v>3228</v>
+        <v>3344</v>
       </c>
     </row>
     <row r="1684" ht="36.0" customHeight="true">
@@ -40683,7 +40689,7 @@
         <v>1683.0</v>
       </c>
       <c r="B1684" t="s" s="3">
-        <v>3344</v>
+        <v>3345</v>
       </c>
       <c r="C1684" t="s" s="2">
         <v>580</v>
@@ -40692,7 +40698,7 @@
         <v>3044</v>
       </c>
       <c r="E1684" t="s" s="3">
-        <v>3345</v>
+        <v>3230</v>
       </c>
     </row>
     <row r="1685" ht="36.0" customHeight="true">
@@ -41281,7 +41287,7 @@
         <v>3414</v>
       </c>
       <c r="C1719" t="s" s="2">
-        <v>751</v>
+        <v>580</v>
       </c>
       <c r="D1719" t="s" s="2">
         <v>3044</v>
@@ -41366,13 +41372,13 @@
         <v>3424</v>
       </c>
       <c r="C1724" t="s" s="2">
-        <v>6</v>
+        <v>751</v>
       </c>
       <c r="D1724" t="s" s="2">
+        <v>3044</v>
+      </c>
+      <c r="E1724" t="s" s="3">
         <v>3425</v>
-      </c>
-      <c r="E1724" t="s" s="3">
-        <v>3426</v>
       </c>
     </row>
     <row r="1725" ht="36.0" customHeight="true">
@@ -41380,13 +41386,13 @@
         <v>1724.0</v>
       </c>
       <c r="B1725" t="s" s="3">
+        <v>3426</v>
+      </c>
+      <c r="C1725" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="D1725" t="s" s="2">
         <v>3427</v>
-      </c>
-      <c r="C1725" t="s" s="2">
-        <v>6</v>
-      </c>
-      <c r="D1725" t="s" s="2">
-        <v>3425</v>
       </c>
       <c r="E1725" t="s" s="3">
         <v>3428</v>
@@ -41403,7 +41409,7 @@
         <v>6</v>
       </c>
       <c r="D1726" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1726" t="s" s="3">
         <v>3430</v>
@@ -41420,7 +41426,7 @@
         <v>6</v>
       </c>
       <c r="D1727" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1727" t="s" s="3">
         <v>3432</v>
@@ -41437,7 +41443,7 @@
         <v>6</v>
       </c>
       <c r="D1728" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1728" t="s" s="3">
         <v>3434</v>
@@ -41454,7 +41460,7 @@
         <v>6</v>
       </c>
       <c r="D1729" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1729" t="s" s="3">
         <v>3436</v>
@@ -41471,7 +41477,7 @@
         <v>6</v>
       </c>
       <c r="D1730" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1730" t="s" s="3">
         <v>3438</v>
@@ -41488,7 +41494,7 @@
         <v>6</v>
       </c>
       <c r="D1731" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1731" t="s" s="3">
         <v>3440</v>
@@ -41505,7 +41511,7 @@
         <v>6</v>
       </c>
       <c r="D1732" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1732" t="s" s="3">
         <v>3442</v>
@@ -41522,7 +41528,7 @@
         <v>6</v>
       </c>
       <c r="D1733" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1733" t="s" s="3">
         <v>3444</v>
@@ -41539,7 +41545,7 @@
         <v>6</v>
       </c>
       <c r="D1734" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1734" t="s" s="3">
         <v>3446</v>
@@ -41556,7 +41562,7 @@
         <v>6</v>
       </c>
       <c r="D1735" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1735" t="s" s="3">
         <v>3448</v>
@@ -41573,7 +41579,7 @@
         <v>6</v>
       </c>
       <c r="D1736" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1736" t="s" s="3">
         <v>3450</v>
@@ -41590,7 +41596,7 @@
         <v>6</v>
       </c>
       <c r="D1737" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1737" t="s" s="3">
         <v>3452</v>
@@ -41607,7 +41613,7 @@
         <v>6</v>
       </c>
       <c r="D1738" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1738" t="s" s="3">
         <v>3454</v>
@@ -41624,7 +41630,7 @@
         <v>6</v>
       </c>
       <c r="D1739" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1739" t="s" s="3">
         <v>3456</v>
@@ -41641,7 +41647,7 @@
         <v>6</v>
       </c>
       <c r="D1740" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1740" t="s" s="3">
         <v>3458</v>
@@ -41658,7 +41664,7 @@
         <v>6</v>
       </c>
       <c r="D1741" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1741" t="s" s="3">
         <v>3460</v>
@@ -41675,7 +41681,7 @@
         <v>6</v>
       </c>
       <c r="D1742" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1742" t="s" s="3">
         <v>3462</v>
@@ -41692,7 +41698,7 @@
         <v>6</v>
       </c>
       <c r="D1743" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1743" t="s" s="3">
         <v>3464</v>
@@ -41709,7 +41715,7 @@
         <v>6</v>
       </c>
       <c r="D1744" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1744" t="s" s="3">
         <v>3466</v>
@@ -41726,7 +41732,7 @@
         <v>6</v>
       </c>
       <c r="D1745" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1745" t="s" s="3">
         <v>3468</v>
@@ -41743,7 +41749,7 @@
         <v>6</v>
       </c>
       <c r="D1746" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1746" t="s" s="3">
         <v>3470</v>
@@ -41760,7 +41766,7 @@
         <v>6</v>
       </c>
       <c r="D1747" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1747" t="s" s="3">
         <v>3472</v>
@@ -41777,7 +41783,7 @@
         <v>6</v>
       </c>
       <c r="D1748" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1748" t="s" s="3">
         <v>3474</v>
@@ -41794,7 +41800,7 @@
         <v>6</v>
       </c>
       <c r="D1749" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1749" t="s" s="3">
         <v>3476</v>
@@ -41811,7 +41817,7 @@
         <v>6</v>
       </c>
       <c r="D1750" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1750" t="s" s="3">
         <v>3478</v>
@@ -41828,7 +41834,7 @@
         <v>6</v>
       </c>
       <c r="D1751" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1751" t="s" s="3">
         <v>3480</v>
@@ -41845,7 +41851,7 @@
         <v>6</v>
       </c>
       <c r="D1752" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1752" t="s" s="3">
         <v>3482</v>
@@ -41862,7 +41868,7 @@
         <v>6</v>
       </c>
       <c r="D1753" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1753" t="s" s="3">
         <v>3484</v>
@@ -41879,7 +41885,7 @@
         <v>6</v>
       </c>
       <c r="D1754" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1754" t="s" s="3">
         <v>3486</v>
@@ -41896,7 +41902,7 @@
         <v>6</v>
       </c>
       <c r="D1755" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1755" t="s" s="3">
         <v>3488</v>
@@ -41913,7 +41919,7 @@
         <v>6</v>
       </c>
       <c r="D1756" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1756" t="s" s="3">
         <v>3490</v>
@@ -41930,7 +41936,7 @@
         <v>6</v>
       </c>
       <c r="D1757" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1757" t="s" s="3">
         <v>3492</v>
@@ -41947,7 +41953,7 @@
         <v>6</v>
       </c>
       <c r="D1758" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1758" t="s" s="3">
         <v>3494</v>
@@ -41964,7 +41970,7 @@
         <v>6</v>
       </c>
       <c r="D1759" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1759" t="s" s="3">
         <v>3496</v>
@@ -41981,7 +41987,7 @@
         <v>6</v>
       </c>
       <c r="D1760" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1760" t="s" s="3">
         <v>3498</v>
@@ -41998,7 +42004,7 @@
         <v>6</v>
       </c>
       <c r="D1761" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1761" t="s" s="3">
         <v>3500</v>
@@ -42015,7 +42021,7 @@
         <v>6</v>
       </c>
       <c r="D1762" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1762" t="s" s="3">
         <v>3502</v>
@@ -42032,7 +42038,7 @@
         <v>6</v>
       </c>
       <c r="D1763" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1763" t="s" s="3">
         <v>3504</v>
@@ -42049,7 +42055,7 @@
         <v>6</v>
       </c>
       <c r="D1764" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1764" t="s" s="3">
         <v>3506</v>
@@ -42066,7 +42072,7 @@
         <v>6</v>
       </c>
       <c r="D1765" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1765" t="s" s="3">
         <v>3508</v>
@@ -42083,7 +42089,7 @@
         <v>6</v>
       </c>
       <c r="D1766" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1766" t="s" s="3">
         <v>3510</v>
@@ -42100,7 +42106,7 @@
         <v>6</v>
       </c>
       <c r="D1767" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1767" t="s" s="3">
         <v>3512</v>
@@ -42117,7 +42123,7 @@
         <v>6</v>
       </c>
       <c r="D1768" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1768" t="s" s="3">
         <v>3514</v>
@@ -42134,7 +42140,7 @@
         <v>6</v>
       </c>
       <c r="D1769" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1769" t="s" s="3">
         <v>3516</v>
@@ -42151,7 +42157,7 @@
         <v>6</v>
       </c>
       <c r="D1770" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1770" t="s" s="3">
         <v>3518</v>
@@ -42165,10 +42171,10 @@
         <v>3519</v>
       </c>
       <c r="C1771" t="s" s="2">
-        <v>580</v>
+        <v>6</v>
       </c>
       <c r="D1771" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1771" t="s" s="3">
         <v>3520</v>
@@ -42185,7 +42191,7 @@
         <v>580</v>
       </c>
       <c r="D1772" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1772" t="s" s="3">
         <v>3522</v>
@@ -42202,7 +42208,7 @@
         <v>580</v>
       </c>
       <c r="D1773" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1773" t="s" s="3">
         <v>3524</v>
@@ -42219,7 +42225,7 @@
         <v>580</v>
       </c>
       <c r="D1774" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1774" t="s" s="3">
         <v>3526</v>
@@ -42236,7 +42242,7 @@
         <v>580</v>
       </c>
       <c r="D1775" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1775" t="s" s="3">
         <v>3528</v>
@@ -42253,7 +42259,7 @@
         <v>580</v>
       </c>
       <c r="D1776" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1776" t="s" s="3">
         <v>3530</v>
@@ -42270,7 +42276,7 @@
         <v>580</v>
       </c>
       <c r="D1777" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1777" t="s" s="3">
         <v>3532</v>
@@ -42287,7 +42293,7 @@
         <v>580</v>
       </c>
       <c r="D1778" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1778" t="s" s="3">
         <v>3534</v>
@@ -42304,7 +42310,7 @@
         <v>580</v>
       </c>
       <c r="D1779" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1779" t="s" s="3">
         <v>3536</v>
@@ -42321,7 +42327,7 @@
         <v>580</v>
       </c>
       <c r="D1780" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1780" t="s" s="3">
         <v>3538</v>
@@ -42338,7 +42344,7 @@
         <v>580</v>
       </c>
       <c r="D1781" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1781" t="s" s="3">
         <v>3540</v>
@@ -42355,7 +42361,7 @@
         <v>580</v>
       </c>
       <c r="D1782" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1782" t="s" s="3">
         <v>3542</v>
@@ -42372,7 +42378,7 @@
         <v>580</v>
       </c>
       <c r="D1783" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1783" t="s" s="3">
         <v>3544</v>
@@ -42389,7 +42395,7 @@
         <v>580</v>
       </c>
       <c r="D1784" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1784" t="s" s="3">
         <v>3546</v>
@@ -42406,7 +42412,7 @@
         <v>580</v>
       </c>
       <c r="D1785" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1785" t="s" s="3">
         <v>3548</v>
@@ -42423,7 +42429,7 @@
         <v>580</v>
       </c>
       <c r="D1786" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1786" t="s" s="3">
         <v>3550</v>
@@ -42440,7 +42446,7 @@
         <v>580</v>
       </c>
       <c r="D1787" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1787" t="s" s="3">
         <v>3552</v>
@@ -42457,7 +42463,7 @@
         <v>580</v>
       </c>
       <c r="D1788" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1788" t="s" s="3">
         <v>3554</v>
@@ -42474,7 +42480,7 @@
         <v>580</v>
       </c>
       <c r="D1789" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1789" t="s" s="3">
         <v>3556</v>
@@ -42491,7 +42497,7 @@
         <v>580</v>
       </c>
       <c r="D1790" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1790" t="s" s="3">
         <v>3558</v>
@@ -42508,7 +42514,7 @@
         <v>580</v>
       </c>
       <c r="D1791" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1791" t="s" s="3">
         <v>3560</v>
@@ -42525,7 +42531,7 @@
         <v>580</v>
       </c>
       <c r="D1792" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1792" t="s" s="3">
         <v>3562</v>
@@ -42542,7 +42548,7 @@
         <v>580</v>
       </c>
       <c r="D1793" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1793" t="s" s="3">
         <v>3564</v>
@@ -42559,7 +42565,7 @@
         <v>580</v>
       </c>
       <c r="D1794" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1794" t="s" s="3">
         <v>3566</v>
@@ -42576,7 +42582,7 @@
         <v>580</v>
       </c>
       <c r="D1795" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1795" t="s" s="3">
         <v>3568</v>
@@ -42593,7 +42599,7 @@
         <v>580</v>
       </c>
       <c r="D1796" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1796" t="s" s="3">
         <v>3570</v>
@@ -42610,7 +42616,7 @@
         <v>580</v>
       </c>
       <c r="D1797" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1797" t="s" s="3">
         <v>3572</v>
@@ -42627,7 +42633,7 @@
         <v>580</v>
       </c>
       <c r="D1798" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1798" t="s" s="3">
         <v>3574</v>
@@ -42644,7 +42650,7 @@
         <v>580</v>
       </c>
       <c r="D1799" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1799" t="s" s="3">
         <v>3576</v>
@@ -42661,7 +42667,7 @@
         <v>580</v>
       </c>
       <c r="D1800" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1800" t="s" s="3">
         <v>3578</v>
@@ -42678,7 +42684,7 @@
         <v>580</v>
       </c>
       <c r="D1801" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1801" t="s" s="3">
         <v>3580</v>
@@ -42695,7 +42701,7 @@
         <v>580</v>
       </c>
       <c r="D1802" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1802" t="s" s="3">
         <v>3582</v>
@@ -42712,7 +42718,7 @@
         <v>580</v>
       </c>
       <c r="D1803" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1803" t="s" s="3">
         <v>3584</v>
@@ -42729,7 +42735,7 @@
         <v>580</v>
       </c>
       <c r="D1804" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1804" t="s" s="3">
         <v>3586</v>
@@ -42743,10 +42749,10 @@
         <v>3587</v>
       </c>
       <c r="C1805" t="s" s="2">
-        <v>751</v>
+        <v>580</v>
       </c>
       <c r="D1805" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1805" t="s" s="3">
         <v>3588</v>
@@ -42763,7 +42769,7 @@
         <v>751</v>
       </c>
       <c r="D1806" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1806" t="s" s="3">
         <v>3590</v>
@@ -42780,7 +42786,7 @@
         <v>751</v>
       </c>
       <c r="D1807" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1807" t="s" s="3">
         <v>3592</v>
@@ -42797,7 +42803,7 @@
         <v>751</v>
       </c>
       <c r="D1808" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1808" t="s" s="3">
         <v>3594</v>
@@ -42814,7 +42820,7 @@
         <v>751</v>
       </c>
       <c r="D1809" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1809" t="s" s="3">
         <v>3596</v>
@@ -42831,7 +42837,7 @@
         <v>751</v>
       </c>
       <c r="D1810" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1810" t="s" s="3">
         <v>3598</v>
@@ -42848,7 +42854,7 @@
         <v>751</v>
       </c>
       <c r="D1811" t="s" s="2">
-        <v>3425</v>
+        <v>3427</v>
       </c>
       <c r="E1811" t="s" s="3">
         <v>3600</v>
@@ -42862,13 +42868,13 @@
         <v>3601</v>
       </c>
       <c r="C1812" t="s" s="2">
-        <v>6</v>
+        <v>751</v>
       </c>
       <c r="D1812" t="s" s="2">
+        <v>3427</v>
+      </c>
+      <c r="E1812" t="s" s="3">
         <v>3602</v>
-      </c>
-      <c r="E1812" t="s" s="3">
-        <v>3603</v>
       </c>
     </row>
     <row r="1813" ht="36.0" customHeight="true">
@@ -42876,13 +42882,13 @@
         <v>1812.0</v>
       </c>
       <c r="B1813" t="s" s="3">
+        <v>3603</v>
+      </c>
+      <c r="C1813" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="D1813" t="s" s="2">
         <v>3604</v>
-      </c>
-      <c r="C1813" t="s" s="2">
-        <v>6</v>
-      </c>
-      <c r="D1813" t="s" s="2">
-        <v>3602</v>
       </c>
       <c r="E1813" t="s" s="3">
         <v>3605</v>
@@ -42899,7 +42905,7 @@
         <v>6</v>
       </c>
       <c r="D1814" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1814" t="s" s="3">
         <v>3607</v>
@@ -42916,7 +42922,7 @@
         <v>6</v>
       </c>
       <c r="D1815" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1815" t="s" s="3">
         <v>3609</v>
@@ -42933,7 +42939,7 @@
         <v>6</v>
       </c>
       <c r="D1816" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1816" t="s" s="3">
         <v>3611</v>
@@ -42950,7 +42956,7 @@
         <v>6</v>
       </c>
       <c r="D1817" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1817" t="s" s="3">
         <v>3613</v>
@@ -42967,7 +42973,7 @@
         <v>6</v>
       </c>
       <c r="D1818" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1818" t="s" s="3">
         <v>3615</v>
@@ -42984,7 +42990,7 @@
         <v>6</v>
       </c>
       <c r="D1819" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1819" t="s" s="3">
         <v>3617</v>
@@ -43001,7 +43007,7 @@
         <v>6</v>
       </c>
       <c r="D1820" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1820" t="s" s="3">
         <v>3619</v>
@@ -43018,7 +43024,7 @@
         <v>6</v>
       </c>
       <c r="D1821" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1821" t="s" s="3">
         <v>3621</v>
@@ -43035,7 +43041,7 @@
         <v>6</v>
       </c>
       <c r="D1822" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1822" t="s" s="3">
         <v>3623</v>
@@ -43052,7 +43058,7 @@
         <v>6</v>
       </c>
       <c r="D1823" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1823" t="s" s="3">
         <v>3625</v>
@@ -43069,7 +43075,7 @@
         <v>6</v>
       </c>
       <c r="D1824" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1824" t="s" s="3">
         <v>3627</v>
@@ -43086,7 +43092,7 @@
         <v>6</v>
       </c>
       <c r="D1825" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1825" t="s" s="3">
         <v>3629</v>
@@ -43103,7 +43109,7 @@
         <v>6</v>
       </c>
       <c r="D1826" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1826" t="s" s="3">
         <v>3631</v>
@@ -43120,7 +43126,7 @@
         <v>6</v>
       </c>
       <c r="D1827" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1827" t="s" s="3">
         <v>3633</v>
@@ -43137,7 +43143,7 @@
         <v>6</v>
       </c>
       <c r="D1828" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1828" t="s" s="3">
         <v>3635</v>
@@ -43154,7 +43160,7 @@
         <v>6</v>
       </c>
       <c r="D1829" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1829" t="s" s="3">
         <v>3637</v>
@@ -43171,7 +43177,7 @@
         <v>6</v>
       </c>
       <c r="D1830" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1830" t="s" s="3">
         <v>3639</v>
@@ -43188,7 +43194,7 @@
         <v>6</v>
       </c>
       <c r="D1831" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1831" t="s" s="3">
         <v>3641</v>
@@ -43205,7 +43211,7 @@
         <v>6</v>
       </c>
       <c r="D1832" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1832" t="s" s="3">
         <v>3643</v>
@@ -43222,7 +43228,7 @@
         <v>6</v>
       </c>
       <c r="D1833" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1833" t="s" s="3">
         <v>3645</v>
@@ -43239,7 +43245,7 @@
         <v>6</v>
       </c>
       <c r="D1834" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1834" t="s" s="3">
         <v>3647</v>
@@ -43256,7 +43262,7 @@
         <v>6</v>
       </c>
       <c r="D1835" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1835" t="s" s="3">
         <v>3649</v>
@@ -43273,7 +43279,7 @@
         <v>6</v>
       </c>
       <c r="D1836" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1836" t="s" s="3">
         <v>3651</v>
@@ -43290,7 +43296,7 @@
         <v>6</v>
       </c>
       <c r="D1837" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1837" t="s" s="3">
         <v>3653</v>
@@ -43307,7 +43313,7 @@
         <v>6</v>
       </c>
       <c r="D1838" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1838" t="s" s="3">
         <v>3655</v>
@@ -43324,7 +43330,7 @@
         <v>6</v>
       </c>
       <c r="D1839" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1839" t="s" s="3">
         <v>3657</v>
@@ -43341,7 +43347,7 @@
         <v>6</v>
       </c>
       <c r="D1840" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1840" t="s" s="3">
         <v>3659</v>
@@ -43358,7 +43364,7 @@
         <v>6</v>
       </c>
       <c r="D1841" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1841" t="s" s="3">
         <v>3661</v>
@@ -43375,7 +43381,7 @@
         <v>6</v>
       </c>
       <c r="D1842" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1842" t="s" s="3">
         <v>3663</v>
@@ -43392,7 +43398,7 @@
         <v>6</v>
       </c>
       <c r="D1843" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1843" t="s" s="3">
         <v>3665</v>
@@ -43409,7 +43415,7 @@
         <v>6</v>
       </c>
       <c r="D1844" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1844" t="s" s="3">
         <v>3667</v>
@@ -43426,7 +43432,7 @@
         <v>6</v>
       </c>
       <c r="D1845" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1845" t="s" s="3">
         <v>3669</v>
@@ -43443,7 +43449,7 @@
         <v>6</v>
       </c>
       <c r="D1846" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1846" t="s" s="3">
         <v>3671</v>
@@ -43460,7 +43466,7 @@
         <v>6</v>
       </c>
       <c r="D1847" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1847" t="s" s="3">
         <v>3673</v>
@@ -43477,7 +43483,7 @@
         <v>6</v>
       </c>
       <c r="D1848" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1848" t="s" s="3">
         <v>3675</v>
@@ -43494,7 +43500,7 @@
         <v>6</v>
       </c>
       <c r="D1849" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1849" t="s" s="3">
         <v>3677</v>
@@ -43511,7 +43517,7 @@
         <v>6</v>
       </c>
       <c r="D1850" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1850" t="s" s="3">
         <v>3679</v>
@@ -43528,7 +43534,7 @@
         <v>6</v>
       </c>
       <c r="D1851" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1851" t="s" s="3">
         <v>3681</v>
@@ -43545,7 +43551,7 @@
         <v>6</v>
       </c>
       <c r="D1852" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1852" t="s" s="3">
         <v>3683</v>
@@ -43562,7 +43568,7 @@
         <v>6</v>
       </c>
       <c r="D1853" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1853" t="s" s="3">
         <v>3685</v>
@@ -43579,7 +43585,7 @@
         <v>6</v>
       </c>
       <c r="D1854" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1854" t="s" s="3">
         <v>3687</v>
@@ -43596,7 +43602,7 @@
         <v>6</v>
       </c>
       <c r="D1855" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1855" t="s" s="3">
         <v>3689</v>
@@ -43613,7 +43619,7 @@
         <v>6</v>
       </c>
       <c r="D1856" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1856" t="s" s="3">
         <v>3691</v>
@@ -43630,7 +43636,7 @@
         <v>6</v>
       </c>
       <c r="D1857" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1857" t="s" s="3">
         <v>3693</v>
@@ -43647,7 +43653,7 @@
         <v>6</v>
       </c>
       <c r="D1858" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1858" t="s" s="3">
         <v>3695</v>
@@ -43664,7 +43670,7 @@
         <v>6</v>
       </c>
       <c r="D1859" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1859" t="s" s="3">
         <v>3697</v>
@@ -43681,7 +43687,7 @@
         <v>6</v>
       </c>
       <c r="D1860" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1860" t="s" s="3">
         <v>3699</v>
@@ -43698,7 +43704,7 @@
         <v>6</v>
       </c>
       <c r="D1861" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1861" t="s" s="3">
         <v>3701</v>
@@ -43715,7 +43721,7 @@
         <v>6</v>
       </c>
       <c r="D1862" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1862" t="s" s="3">
         <v>3703</v>
@@ -43732,7 +43738,7 @@
         <v>6</v>
       </c>
       <c r="D1863" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1863" t="s" s="3">
         <v>3705</v>
@@ -43749,7 +43755,7 @@
         <v>6</v>
       </c>
       <c r="D1864" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1864" t="s" s="3">
         <v>3707</v>
@@ -43766,7 +43772,7 @@
         <v>6</v>
       </c>
       <c r="D1865" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1865" t="s" s="3">
         <v>3709</v>
@@ -43783,7 +43789,7 @@
         <v>6</v>
       </c>
       <c r="D1866" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1866" t="s" s="3">
         <v>3711</v>
@@ -43800,7 +43806,7 @@
         <v>6</v>
       </c>
       <c r="D1867" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1867" t="s" s="3">
         <v>3713</v>
@@ -43817,7 +43823,7 @@
         <v>6</v>
       </c>
       <c r="D1868" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1868" t="s" s="3">
         <v>3715</v>
@@ -43834,7 +43840,7 @@
         <v>6</v>
       </c>
       <c r="D1869" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1869" t="s" s="3">
         <v>3717</v>
@@ -43851,7 +43857,7 @@
         <v>6</v>
       </c>
       <c r="D1870" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1870" t="s" s="3">
         <v>3719</v>
@@ -43868,7 +43874,7 @@
         <v>6</v>
       </c>
       <c r="D1871" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1871" t="s" s="3">
         <v>3721</v>
@@ -43885,7 +43891,7 @@
         <v>6</v>
       </c>
       <c r="D1872" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1872" t="s" s="3">
         <v>3723</v>
@@ -43902,7 +43908,7 @@
         <v>6</v>
       </c>
       <c r="D1873" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1873" t="s" s="3">
         <v>3725</v>
@@ -43919,7 +43925,7 @@
         <v>6</v>
       </c>
       <c r="D1874" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1874" t="s" s="3">
         <v>3727</v>
@@ -43936,7 +43942,7 @@
         <v>6</v>
       </c>
       <c r="D1875" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1875" t="s" s="3">
         <v>3729</v>
@@ -43953,7 +43959,7 @@
         <v>6</v>
       </c>
       <c r="D1876" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1876" t="s" s="3">
         <v>3731</v>
@@ -43970,7 +43976,7 @@
         <v>6</v>
       </c>
       <c r="D1877" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1877" t="s" s="3">
         <v>3733</v>
@@ -43987,7 +43993,7 @@
         <v>6</v>
       </c>
       <c r="D1878" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1878" t="s" s="3">
         <v>3735</v>
@@ -44004,7 +44010,7 @@
         <v>6</v>
       </c>
       <c r="D1879" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1879" t="s" s="3">
         <v>3737</v>
@@ -44021,7 +44027,7 @@
         <v>6</v>
       </c>
       <c r="D1880" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1880" t="s" s="3">
         <v>3739</v>
@@ -44038,7 +44044,7 @@
         <v>6</v>
       </c>
       <c r="D1881" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1881" t="s" s="3">
         <v>3741</v>
@@ -44055,7 +44061,7 @@
         <v>6</v>
       </c>
       <c r="D1882" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1882" t="s" s="3">
         <v>3743</v>
@@ -44072,7 +44078,7 @@
         <v>6</v>
       </c>
       <c r="D1883" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1883" t="s" s="3">
         <v>3745</v>
@@ -44089,7 +44095,7 @@
         <v>6</v>
       </c>
       <c r="D1884" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1884" t="s" s="3">
         <v>3747</v>
@@ -44106,7 +44112,7 @@
         <v>6</v>
       </c>
       <c r="D1885" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1885" t="s" s="3">
         <v>3749</v>
@@ -44123,7 +44129,7 @@
         <v>6</v>
       </c>
       <c r="D1886" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1886" t="s" s="3">
         <v>3751</v>
@@ -44140,7 +44146,7 @@
         <v>6</v>
       </c>
       <c r="D1887" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1887" t="s" s="3">
         <v>3753</v>
@@ -44157,7 +44163,7 @@
         <v>6</v>
       </c>
       <c r="D1888" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1888" t="s" s="3">
         <v>3755</v>
@@ -44174,7 +44180,7 @@
         <v>6</v>
       </c>
       <c r="D1889" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1889" t="s" s="3">
         <v>3757</v>
@@ -44191,7 +44197,7 @@
         <v>6</v>
       </c>
       <c r="D1890" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1890" t="s" s="3">
         <v>3759</v>
@@ -44208,7 +44214,7 @@
         <v>6</v>
       </c>
       <c r="D1891" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1891" t="s" s="3">
         <v>3761</v>
@@ -44225,7 +44231,7 @@
         <v>6</v>
       </c>
       <c r="D1892" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1892" t="s" s="3">
         <v>3763</v>
@@ -44242,7 +44248,7 @@
         <v>6</v>
       </c>
       <c r="D1893" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1893" t="s" s="3">
         <v>3765</v>
@@ -44259,7 +44265,7 @@
         <v>6</v>
       </c>
       <c r="D1894" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1894" t="s" s="3">
         <v>3767</v>
@@ -44276,7 +44282,7 @@
         <v>6</v>
       </c>
       <c r="D1895" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1895" t="s" s="3">
         <v>3769</v>
@@ -44293,7 +44299,7 @@
         <v>6</v>
       </c>
       <c r="D1896" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1896" t="s" s="3">
         <v>3771</v>
@@ -44310,7 +44316,7 @@
         <v>6</v>
       </c>
       <c r="D1897" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1897" t="s" s="3">
         <v>3773</v>
@@ -44327,7 +44333,7 @@
         <v>6</v>
       </c>
       <c r="D1898" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1898" t="s" s="3">
         <v>3775</v>
@@ -44344,7 +44350,7 @@
         <v>6</v>
       </c>
       <c r="D1899" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1899" t="s" s="3">
         <v>3777</v>
@@ -44361,7 +44367,7 @@
         <v>6</v>
       </c>
       <c r="D1900" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1900" t="s" s="3">
         <v>3779</v>
@@ -44378,7 +44384,7 @@
         <v>6</v>
       </c>
       <c r="D1901" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1901" t="s" s="3">
         <v>3781</v>
@@ -44395,7 +44401,7 @@
         <v>6</v>
       </c>
       <c r="D1902" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1902" t="s" s="3">
         <v>3783</v>
@@ -44412,7 +44418,7 @@
         <v>6</v>
       </c>
       <c r="D1903" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1903" t="s" s="3">
         <v>3785</v>
@@ -44429,7 +44435,7 @@
         <v>6</v>
       </c>
       <c r="D1904" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1904" t="s" s="3">
         <v>3787</v>
@@ -44446,7 +44452,7 @@
         <v>6</v>
       </c>
       <c r="D1905" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1905" t="s" s="3">
         <v>3789</v>
@@ -44463,7 +44469,7 @@
         <v>6</v>
       </c>
       <c r="D1906" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1906" t="s" s="3">
         <v>3791</v>
@@ -44480,7 +44486,7 @@
         <v>6</v>
       </c>
       <c r="D1907" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1907" t="s" s="3">
         <v>3793</v>
@@ -44497,7 +44503,7 @@
         <v>6</v>
       </c>
       <c r="D1908" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1908" t="s" s="3">
         <v>3795</v>
@@ -44514,7 +44520,7 @@
         <v>6</v>
       </c>
       <c r="D1909" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1909" t="s" s="3">
         <v>3797</v>
@@ -44531,7 +44537,7 @@
         <v>6</v>
       </c>
       <c r="D1910" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1910" t="s" s="3">
         <v>3799</v>
@@ -44548,7 +44554,7 @@
         <v>6</v>
       </c>
       <c r="D1911" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1911" t="s" s="3">
         <v>3801</v>
@@ -44559,16 +44565,16 @@
         <v>1911.0</v>
       </c>
       <c r="B1912" t="s" s="3">
-        <v>2275</v>
+        <v>3802</v>
       </c>
       <c r="C1912" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D1912" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1912" t="s" s="3">
-        <v>3802</v>
+        <v>3803</v>
       </c>
     </row>
     <row r="1913" ht="36.0" customHeight="true">
@@ -44576,13 +44582,13 @@
         <v>1912.0</v>
       </c>
       <c r="B1913" t="s" s="3">
-        <v>3803</v>
+        <v>2275</v>
       </c>
       <c r="C1913" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D1913" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1913" t="s" s="3">
         <v>3804</v>
@@ -44599,7 +44605,7 @@
         <v>6</v>
       </c>
       <c r="D1914" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1914" t="s" s="3">
         <v>3806</v>
@@ -44616,7 +44622,7 @@
         <v>6</v>
       </c>
       <c r="D1915" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1915" t="s" s="3">
         <v>3808</v>
@@ -44633,7 +44639,7 @@
         <v>6</v>
       </c>
       <c r="D1916" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1916" t="s" s="3">
         <v>3810</v>
@@ -44650,7 +44656,7 @@
         <v>6</v>
       </c>
       <c r="D1917" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1917" t="s" s="3">
         <v>3812</v>
@@ -44667,7 +44673,7 @@
         <v>6</v>
       </c>
       <c r="D1918" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1918" t="s" s="3">
         <v>3814</v>
@@ -44684,7 +44690,7 @@
         <v>6</v>
       </c>
       <c r="D1919" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1919" t="s" s="3">
         <v>3816</v>
@@ -44701,7 +44707,7 @@
         <v>6</v>
       </c>
       <c r="D1920" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1920" t="s" s="3">
         <v>3818</v>
@@ -44715,10 +44721,10 @@
         <v>3819</v>
       </c>
       <c r="C1921" t="s" s="2">
-        <v>580</v>
+        <v>6</v>
       </c>
       <c r="D1921" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1921" t="s" s="3">
         <v>3820</v>
@@ -44735,7 +44741,7 @@
         <v>580</v>
       </c>
       <c r="D1922" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1922" t="s" s="3">
         <v>3822</v>
@@ -44752,7 +44758,7 @@
         <v>580</v>
       </c>
       <c r="D1923" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1923" t="s" s="3">
         <v>3824</v>
@@ -44769,7 +44775,7 @@
         <v>580</v>
       </c>
       <c r="D1924" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1924" t="s" s="3">
         <v>3826</v>
@@ -44786,7 +44792,7 @@
         <v>580</v>
       </c>
       <c r="D1925" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1925" t="s" s="3">
         <v>3828</v>
@@ -44803,7 +44809,7 @@
         <v>580</v>
       </c>
       <c r="D1926" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1926" t="s" s="3">
         <v>3830</v>
@@ -44820,7 +44826,7 @@
         <v>580</v>
       </c>
       <c r="D1927" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1927" t="s" s="3">
         <v>3832</v>
@@ -44837,7 +44843,7 @@
         <v>580</v>
       </c>
       <c r="D1928" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1928" t="s" s="3">
         <v>3834</v>
@@ -44854,7 +44860,7 @@
         <v>580</v>
       </c>
       <c r="D1929" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1929" t="s" s="3">
         <v>3836</v>
@@ -44871,7 +44877,7 @@
         <v>580</v>
       </c>
       <c r="D1930" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1930" t="s" s="3">
         <v>3838</v>
@@ -44888,7 +44894,7 @@
         <v>580</v>
       </c>
       <c r="D1931" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1931" t="s" s="3">
         <v>3840</v>
@@ -44905,7 +44911,7 @@
         <v>580</v>
       </c>
       <c r="D1932" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1932" t="s" s="3">
         <v>3842</v>
@@ -44922,7 +44928,7 @@
         <v>580</v>
       </c>
       <c r="D1933" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1933" t="s" s="3">
         <v>3844</v>
@@ -44939,7 +44945,7 @@
         <v>580</v>
       </c>
       <c r="D1934" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1934" t="s" s="3">
         <v>3846</v>
@@ -44956,7 +44962,7 @@
         <v>580</v>
       </c>
       <c r="D1935" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1935" t="s" s="3">
         <v>3848</v>
@@ -44973,7 +44979,7 @@
         <v>580</v>
       </c>
       <c r="D1936" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1936" t="s" s="3">
         <v>3850</v>
@@ -44990,7 +44996,7 @@
         <v>580</v>
       </c>
       <c r="D1937" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1937" t="s" s="3">
         <v>3852</v>
@@ -45007,7 +45013,7 @@
         <v>580</v>
       </c>
       <c r="D1938" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1938" t="s" s="3">
         <v>3854</v>
@@ -45024,7 +45030,7 @@
         <v>580</v>
       </c>
       <c r="D1939" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1939" t="s" s="3">
         <v>3856</v>
@@ -45041,7 +45047,7 @@
         <v>580</v>
       </c>
       <c r="D1940" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1940" t="s" s="3">
         <v>3858</v>
@@ -45058,7 +45064,7 @@
         <v>580</v>
       </c>
       <c r="D1941" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1941" t="s" s="3">
         <v>3860</v>
@@ -45075,7 +45081,7 @@
         <v>580</v>
       </c>
       <c r="D1942" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1942" t="s" s="3">
         <v>3862</v>
@@ -45092,7 +45098,7 @@
         <v>580</v>
       </c>
       <c r="D1943" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1943" t="s" s="3">
         <v>3864</v>
@@ -45109,7 +45115,7 @@
         <v>580</v>
       </c>
       <c r="D1944" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1944" t="s" s="3">
         <v>3866</v>
@@ -45126,7 +45132,7 @@
         <v>580</v>
       </c>
       <c r="D1945" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1945" t="s" s="3">
         <v>3868</v>
@@ -45143,7 +45149,7 @@
         <v>580</v>
       </c>
       <c r="D1946" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1946" t="s" s="3">
         <v>3870</v>
@@ -45160,7 +45166,7 @@
         <v>580</v>
       </c>
       <c r="D1947" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1947" t="s" s="3">
         <v>3872</v>
@@ -45177,7 +45183,7 @@
         <v>580</v>
       </c>
       <c r="D1948" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1948" t="s" s="3">
         <v>3874</v>
@@ -45194,7 +45200,7 @@
         <v>580</v>
       </c>
       <c r="D1949" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1949" t="s" s="3">
         <v>3876</v>
@@ -45211,7 +45217,7 @@
         <v>580</v>
       </c>
       <c r="D1950" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1950" t="s" s="3">
         <v>3878</v>
@@ -45228,7 +45234,7 @@
         <v>580</v>
       </c>
       <c r="D1951" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1951" t="s" s="3">
         <v>3880</v>
@@ -45245,7 +45251,7 @@
         <v>580</v>
       </c>
       <c r="D1952" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1952" t="s" s="3">
         <v>3882</v>
@@ -45262,7 +45268,7 @@
         <v>580</v>
       </c>
       <c r="D1953" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1953" t="s" s="3">
         <v>3884</v>
@@ -45279,10 +45285,10 @@
         <v>580</v>
       </c>
       <c r="D1954" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1954" t="s" s="3">
-        <v>3649</v>
+        <v>3886</v>
       </c>
     </row>
     <row r="1955" ht="36.0" customHeight="true">
@@ -45290,16 +45296,16 @@
         <v>1954.0</v>
       </c>
       <c r="B1955" t="s" s="3">
-        <v>3886</v>
+        <v>3887</v>
       </c>
       <c r="C1955" t="s" s="2">
         <v>580</v>
       </c>
       <c r="D1955" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1955" t="s" s="3">
-        <v>3887</v>
+        <v>3651</v>
       </c>
     </row>
     <row r="1956" ht="36.0" customHeight="true">
@@ -45313,7 +45319,7 @@
         <v>580</v>
       </c>
       <c r="D1956" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1956" t="s" s="3">
         <v>3889</v>
@@ -45330,7 +45336,7 @@
         <v>580</v>
       </c>
       <c r="D1957" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1957" t="s" s="3">
         <v>3891</v>
@@ -45347,7 +45353,7 @@
         <v>580</v>
       </c>
       <c r="D1958" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1958" t="s" s="3">
         <v>3893</v>
@@ -45361,10 +45367,10 @@
         <v>3894</v>
       </c>
       <c r="C1959" t="s" s="2">
-        <v>751</v>
+        <v>580</v>
       </c>
       <c r="D1959" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1959" t="s" s="3">
         <v>3895</v>
@@ -45381,7 +45387,7 @@
         <v>751</v>
       </c>
       <c r="D1960" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1960" t="s" s="3">
         <v>3897</v>
@@ -45392,16 +45398,16 @@
         <v>1960.0</v>
       </c>
       <c r="B1961" t="s" s="3">
-        <v>3881</v>
+        <v>3898</v>
       </c>
       <c r="C1961" t="s" s="2">
         <v>751</v>
       </c>
       <c r="D1961" t="s" s="2">
-        <v>3602</v>
+        <v>3604</v>
       </c>
       <c r="E1961" t="s" s="3">
-        <v>3898</v>
+        <v>3899</v>
       </c>
     </row>
     <row r="1962" ht="36.0" customHeight="true">
@@ -45409,16 +45415,16 @@
         <v>1961.0</v>
       </c>
       <c r="B1962" t="s" s="3">
-        <v>3899</v>
+        <v>3883</v>
       </c>
       <c r="C1962" t="s" s="2">
-        <v>6</v>
+        <v>751</v>
       </c>
       <c r="D1962" t="s" s="2">
+        <v>3604</v>
+      </c>
+      <c r="E1962" t="s" s="3">
         <v>3900</v>
-      </c>
-      <c r="E1962" t="s" s="3">
-        <v>3901</v>
       </c>
     </row>
     <row r="1963" ht="36.0" customHeight="true">
@@ -45426,13 +45432,13 @@
         <v>1962.0</v>
       </c>
       <c r="B1963" t="s" s="3">
+        <v>3901</v>
+      </c>
+      <c r="C1963" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="D1963" t="s" s="2">
         <v>3902</v>
-      </c>
-      <c r="C1963" t="s" s="2">
-        <v>6</v>
-      </c>
-      <c r="D1963" t="s" s="2">
-        <v>3900</v>
       </c>
       <c r="E1963" t="s" s="3">
         <v>3903</v>
@@ -45449,7 +45455,7 @@
         <v>6</v>
       </c>
       <c r="D1964" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1964" t="s" s="3">
         <v>3905</v>
@@ -45466,7 +45472,7 @@
         <v>6</v>
       </c>
       <c r="D1965" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1965" t="s" s="3">
         <v>3907</v>
@@ -45483,7 +45489,7 @@
         <v>6</v>
       </c>
       <c r="D1966" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1966" t="s" s="3">
         <v>3909</v>
@@ -45500,7 +45506,7 @@
         <v>6</v>
       </c>
       <c r="D1967" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1967" t="s" s="3">
         <v>3911</v>
@@ -45517,7 +45523,7 @@
         <v>6</v>
       </c>
       <c r="D1968" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1968" t="s" s="3">
         <v>3913</v>
@@ -45534,7 +45540,7 @@
         <v>6</v>
       </c>
       <c r="D1969" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1969" t="s" s="3">
         <v>3915</v>
@@ -45551,7 +45557,7 @@
         <v>6</v>
       </c>
       <c r="D1970" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1970" t="s" s="3">
         <v>3917</v>
@@ -45568,7 +45574,7 @@
         <v>6</v>
       </c>
       <c r="D1971" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1971" t="s" s="3">
         <v>3919</v>
@@ -45585,7 +45591,7 @@
         <v>6</v>
       </c>
       <c r="D1972" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1972" t="s" s="3">
         <v>3921</v>
@@ -45602,7 +45608,7 @@
         <v>6</v>
       </c>
       <c r="D1973" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1973" t="s" s="3">
         <v>3923</v>
@@ -45619,7 +45625,7 @@
         <v>6</v>
       </c>
       <c r="D1974" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1974" t="s" s="3">
         <v>3925</v>
@@ -45636,7 +45642,7 @@
         <v>6</v>
       </c>
       <c r="D1975" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1975" t="s" s="3">
         <v>3927</v>
@@ -45653,7 +45659,7 @@
         <v>6</v>
       </c>
       <c r="D1976" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1976" t="s" s="3">
         <v>3929</v>
@@ -45670,7 +45676,7 @@
         <v>6</v>
       </c>
       <c r="D1977" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1977" t="s" s="3">
         <v>3931</v>
@@ -45687,7 +45693,7 @@
         <v>6</v>
       </c>
       <c r="D1978" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1978" t="s" s="3">
         <v>3933</v>
@@ -45704,7 +45710,7 @@
         <v>6</v>
       </c>
       <c r="D1979" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1979" t="s" s="3">
         <v>3935</v>
@@ -45721,7 +45727,7 @@
         <v>6</v>
       </c>
       <c r="D1980" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1980" t="s" s="3">
         <v>3937</v>
@@ -45738,7 +45744,7 @@
         <v>6</v>
       </c>
       <c r="D1981" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1981" t="s" s="3">
         <v>3939</v>
@@ -45755,7 +45761,7 @@
         <v>6</v>
       </c>
       <c r="D1982" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1982" t="s" s="3">
         <v>3941</v>
@@ -45772,7 +45778,7 @@
         <v>6</v>
       </c>
       <c r="D1983" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1983" t="s" s="3">
         <v>3943</v>
@@ -45789,7 +45795,7 @@
         <v>6</v>
       </c>
       <c r="D1984" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1984" t="s" s="3">
         <v>3945</v>
@@ -45806,7 +45812,7 @@
         <v>6</v>
       </c>
       <c r="D1985" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1985" t="s" s="3">
         <v>3947</v>
@@ -45823,7 +45829,7 @@
         <v>6</v>
       </c>
       <c r="D1986" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1986" t="s" s="3">
         <v>3949</v>
@@ -45840,7 +45846,7 @@
         <v>6</v>
       </c>
       <c r="D1987" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1987" t="s" s="3">
         <v>3951</v>
@@ -45857,7 +45863,7 @@
         <v>6</v>
       </c>
       <c r="D1988" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1988" t="s" s="3">
         <v>3953</v>
@@ -45871,13 +45877,13 @@
         <v>3954</v>
       </c>
       <c r="C1989" t="s" s="2">
-        <v>580</v>
+        <v>6</v>
       </c>
       <c r="D1989" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1989" t="s" s="3">
-        <v>3935</v>
+        <v>3955</v>
       </c>
     </row>
     <row r="1990" ht="36.0" customHeight="true">
@@ -45885,16 +45891,16 @@
         <v>1989.0</v>
       </c>
       <c r="B1990" t="s" s="3">
-        <v>3955</v>
+        <v>3956</v>
       </c>
       <c r="C1990" t="s" s="2">
         <v>580</v>
       </c>
       <c r="D1990" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1990" t="s" s="3">
-        <v>3956</v>
+        <v>3937</v>
       </c>
     </row>
     <row r="1991" ht="36.0" customHeight="true">
@@ -45908,7 +45914,7 @@
         <v>580</v>
       </c>
       <c r="D1991" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1991" t="s" s="3">
         <v>3958</v>
@@ -45925,7 +45931,7 @@
         <v>580</v>
       </c>
       <c r="D1992" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1992" t="s" s="3">
         <v>3960</v>
@@ -45942,7 +45948,7 @@
         <v>580</v>
       </c>
       <c r="D1993" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1993" t="s" s="3">
         <v>3962</v>
@@ -45959,7 +45965,7 @@
         <v>580</v>
       </c>
       <c r="D1994" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1994" t="s" s="3">
         <v>3964</v>
@@ -45976,7 +45982,7 @@
         <v>580</v>
       </c>
       <c r="D1995" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1995" t="s" s="3">
         <v>3966</v>
@@ -45993,7 +45999,7 @@
         <v>580</v>
       </c>
       <c r="D1996" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1996" t="s" s="3">
         <v>3968</v>
@@ -46010,7 +46016,7 @@
         <v>580</v>
       </c>
       <c r="D1997" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1997" t="s" s="3">
         <v>3970</v>
@@ -46027,7 +46033,7 @@
         <v>580</v>
       </c>
       <c r="D1998" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1998" t="s" s="3">
         <v>3972</v>
@@ -46044,7 +46050,7 @@
         <v>580</v>
       </c>
       <c r="D1999" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E1999" t="s" s="3">
         <v>3974</v>
@@ -46061,7 +46067,7 @@
         <v>580</v>
       </c>
       <c r="D2000" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E2000" t="s" s="3">
         <v>3976</v>
@@ -46078,7 +46084,7 @@
         <v>580</v>
       </c>
       <c r="D2001" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E2001" t="s" s="3">
         <v>3978</v>
@@ -46095,7 +46101,7 @@
         <v>580</v>
       </c>
       <c r="D2002" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E2002" t="s" s="3">
         <v>3980</v>
@@ -46112,7 +46118,7 @@
         <v>580</v>
       </c>
       <c r="D2003" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E2003" t="s" s="3">
         <v>3982</v>
@@ -46129,10 +46135,27 @@
         <v>580</v>
       </c>
       <c r="D2004" t="s" s="2">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="E2004" t="s" s="3">
         <v>3984</v>
+      </c>
+    </row>
+    <row r="2005" ht="36.0" customHeight="true">
+      <c r="A2005" t="n" s="2">
+        <v>2004.0</v>
+      </c>
+      <c r="B2005" t="s" s="3">
+        <v>3985</v>
+      </c>
+      <c r="C2005" t="s" s="2">
+        <v>580</v>
+      </c>
+      <c r="D2005" t="s" s="2">
+        <v>3902</v>
+      </c>
+      <c r="E2005" t="s" s="3">
+        <v>3986</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
로봇 자동 갱신: 2026-05-30
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3734,12 +3734,12 @@
     <t>조선백호</t>
   </si>
   <si>
+    <t>인천광역시 중구 개항로96번길 11(1층 경동)</t>
+  </si>
+  <si>
     <t>인천광역시 중구 개항로96번길 11(1,2층 경동)</t>
   </si>
   <si>
-    <t>인천광역시 중구 개항로96번길 11(1층 경동)</t>
-  </si>
-  <si>
     <t>주윤 상차림</t>
   </si>
   <si>
@@ -3881,10 +3881,10 @@
     <t>그리너리 바스켓</t>
   </si>
   <si>
+    <t>인천광역시 중구 백운로 510(1동 지1층 운북동)</t>
+  </si>
+  <si>
     <t>인천광역시 중구 백운로 510(2동 1,2층 운북동)</t>
-  </si>
-  <si>
-    <t>인천광역시 중구 백운로 510(1동 지1층 운북동)</t>
   </si>
   <si>
     <t>꿈꾸는카페-혜윰도그파크점</t>

</xml_diff>

<commit_message>
로봇 자동 갱신: 2026-06-21
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4073,10 +4073,10 @@
     <t>그리너리 바스켓</t>
   </si>
   <si>
+    <t>인천광역시 중구 백운로 510(1동 지1층 운북동)</t>
+  </si>
+  <si>
     <t>인천광역시 중구 백운로 510(2동 1,2층 운북동)</t>
-  </si>
-  <si>
-    <t>인천광역시 중구 백운로 510(1동 지1층 운북동)</t>
   </si>
   <si>
     <t>꽁냥이네</t>

</xml_diff>

<commit_message>
로봇 자동 갱신: 2026-08-09
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5342,10 +5342,10 @@
     <t>그리너리 바스켓</t>
   </si>
   <si>
+    <t>인천광역시 영종구 백운로 510(1동 지1층 운북동)</t>
+  </si>
+  <si>
     <t>인천광역시 영종구 백운로 510(2동 1,2층 운북동)</t>
-  </si>
-  <si>
-    <t>인천광역시 영종구 백운로 510(1동 지1층 운북동)</t>
   </si>
   <si>
     <t>꽁냥이네</t>

</xml_diff>